<commit_message>
Updated the co ordinates and UI for routes page
</commit_message>
<xml_diff>
--- a/backend/Fare Matrix.xlsx
+++ b/backend/Fare Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Coding\Projects\Metro_React JS\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Coding\Projects\Ahmedabad Metro\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175BBAC1-E063-4436-A9F9-704A556D5826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E965954C-D31C-4170-905C-D9C40983E605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F605D172-C8CF-4215-BA16-067A9175F1B0}"/>
   </bookViews>
@@ -204,7 +204,7 @@
     <t>Sector-10A</t>
   </si>
   <si>
-    <t>GIFT City</t>
+    <t>Gift City</t>
   </si>
 </sst>
 </file>

</xml_diff>